<commit_message>
fix(eval): confirm 8 gold_pending rows + polish real_014
User confirmed the empty preferred_skills on real_005/010/011/014/027/
037/038/040 are genuine (JDs have no preferred section), so mark them
gold_pending=false. build script now preserves hand-confirmed flags
across rebuilds (previously recomputed from the auto rule on every
build). real_014 English gold rebuilt from the JD bullets (4 required /
5 responsibilities) instead of raw newline fragments; splitter now
splits newline-delimited cells on newlines only, keeping sentences with
commas/slashes intact while comma-separated single-line lists still split.
Real-corpus baseline unchanged (span 0, UNKNOWN 28.7%, ATS 100%).
</commit_message>
<xml_diff>
--- a/evaluation/datasets/real_jd_cases_completed.xlsx
+++ b/evaluation/datasets/real_jd_cases_completed.xlsx
@@ -2320,22 +2320,20 @@
       <c r="E16" s="9" t="inlineStr"/>
       <c r="F16" s="9" t="inlineStr">
         <is>
-          <t>Qualifications
-To be successful in the role, you should meet the followingrequirements:
--Strong verbal and written communication skills and solidexperience in face-to-face presentation
--Strong Excel, PowerPoint, and MS Word skills.
--Engaging and influencing withCustomers/Stakeholders/Colleagues- Excellent analytical and problem-solving skills, proposingsolutions when escalating.</t>
+          <t>Strong verbal and written communication skills and solid experience in face-to-face presentation
+Strong Excel, PowerPoint, and MS Word skills
+Engaging and influencing with Customers/Stakeholders/Colleagues
+Excellent analytical and problem-solving skills, proposing solutions when escalating</t>
         </is>
       </c>
       <c r="G16" s="9" t="inlineStr"/>
       <c r="H16" s="9" t="inlineStr">
         <is>
-          <t>In this role, you will:
--Oversees development of a project plans and recommendsmeasures to optimize the plan making it more effort, time andcost effective.
--Collaborate closely with the team to define the project scope,objectives, requirements, and timeline.
--Demonstrates working knowledge of Programme /ProjectFramework, supporting the creation of detailed plans includingkey activities and milestones
--Has good knowledge of risks/issues/dependenciesmanagement techniques.
--Takes ownership of problems and escalates when needed(remaining calm, knowing when to escalate, escalates withpossible solutions)</t>
+          <t>Oversees development of a project plans and recommends measures to optimize the plan making it more effort, time and cost effective
+Collaborate closely with the team to define the project scope, objectives, requirements, and timeline
+Demonstrates working knowledge of Programme/Project Framework, supporting the creation of detailed plans including key activities and milestones
+Has good knowledge of risks/issues/dependencies management techniques
+Takes ownership of problems and escalates when needed (remaining calm, knowing when to escalate, escalates with possible solutions)</t>
         </is>
       </c>
       <c r="I16" s="9" t="inlineStr"/>

</xml_diff>